<commit_message>
add test plan for 5.2
</commit_message>
<xml_diff>
--- a/Lab5_EC.xlsx
+++ b/Lab5_EC.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\SQA\Lab5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16674CBF-08A4-48BE-AB12-B9B10560941C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E1564C1-9AE0-46A5-8F11-E60B7241B9E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{2D3B1ECF-CE0B-884D-A6E2-5EDB198A06FE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{2D3B1ECF-CE0B-884D-A6E2-5EDB198A06FE}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Summary" sheetId="4" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="132">
   <si>
     <t>Test Case Design and Test Results</t>
   </si>
@@ -132,24 +132,6 @@
     <t>Total</t>
   </si>
   <si>
-    <t>TC001</t>
-  </si>
-  <si>
-    <t>TC002</t>
-  </si>
-  <si>
-    <t>TC003</t>
-  </si>
-  <si>
-    <t>TC004</t>
-  </si>
-  <si>
-    <t>TC005</t>
-  </si>
-  <si>
-    <t>TC006</t>
-  </si>
-  <si>
     <t>TC007</t>
   </si>
   <si>
@@ -349,6 +331,111 @@
   </si>
   <si>
     <t>assurance</t>
+  </si>
+  <si>
+    <t>ค่าscore 1 มีค่ามากที่สุด</t>
+  </si>
+  <si>
+    <t>ค่าscore 2 มีค่ามากที่สุด</t>
+  </si>
+  <si>
+    <t>ค่าscore 3 มีค่ามากที่สุด</t>
+  </si>
+  <si>
+    <t>มีscore ค่าใดค่าหนึ่งไม่อยู่ในช่วงที่กำหนด 0-500</t>
+  </si>
+  <si>
+    <t>ค่าที่รับมีจำนวนมากกว่า 3 ค่า</t>
+  </si>
+  <si>
+    <t>มีค่าสูงสุดอย่างน้อยสองค่าที่เท่ากัน</t>
+  </si>
+  <si>
+    <t>TC001 EC1</t>
+  </si>
+  <si>
+    <t>ค่าที่รับมามีจำนวนน้อยกว่า 3 ค่า</t>
+  </si>
+  <si>
+    <t>TC002 EC2</t>
+  </si>
+  <si>
+    <t>TC003 EC3</t>
+  </si>
+  <si>
+    <t>TC004 EC4</t>
+  </si>
+  <si>
+    <t>TC005 EC5</t>
+  </si>
+  <si>
+    <t>TC006 EC6</t>
+  </si>
+  <si>
+    <t>TC007 EC7</t>
+  </si>
+  <si>
+    <t>Expected Result (3 argument)</t>
+  </si>
+  <si>
+    <t>Actual Result (3 argument)</t>
+  </si>
+  <si>
+    <t>Expected Result (Array)</t>
+  </si>
+  <si>
+    <t>Actual Result (Array)</t>
+  </si>
+  <si>
+    <t>Score out of bound</t>
+  </si>
+  <si>
+    <t>Attempt Over than 3</t>
+  </si>
+  <si>
+    <t>Attempt Lower than 3</t>
+  </si>
+  <si>
+    <t>250, 100, 150</t>
+  </si>
+  <si>
+    <t>{250, 100, 150}</t>
+  </si>
+  <si>
+    <t>1000, -1, 250</t>
+  </si>
+  <si>
+    <t>100, 300, 275</t>
+  </si>
+  <si>
+    <t>{100, 300, 275</t>
+  </si>
+  <si>
+    <t>100, 250, 500</t>
+  </si>
+  <si>
+    <t>{100, 250, 500}</t>
+  </si>
+  <si>
+    <t>11 , 12</t>
+  </si>
+  <si>
+    <t>1, 2, 3, 4</t>
+  </si>
+  <si>
+    <t>200 ,200, 135</t>
+  </si>
+  <si>
+    <t>{200 ,200, 135}</t>
+  </si>
+  <si>
+    <t>{1000, -1, 250}</t>
+  </si>
+  <si>
+    <t>{1, 2, 3, 4}</t>
+  </si>
+  <si>
+    <t>{11 , 12}</t>
   </si>
 </sst>
 </file>
@@ -653,7 +740,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -723,14 +810,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -749,30 +830,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -797,7 +854,56 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1149,7 +1255,7 @@
   <sheetData>
     <row r="2" spans="1:7" ht="54" x14ac:dyDescent="0.75">
       <c r="A2" s="8" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>23</v>
@@ -1172,7 +1278,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.75">
       <c r="A3" s="28" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -1183,7 +1289,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.75">
       <c r="A4" s="28" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -1194,7 +1300,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.75">
       <c r="A5" s="28" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -1246,134 +1352,134 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="46" t="s">
-        <v>43</v>
-      </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="47"/>
+      <c r="A1" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="37"/>
     </row>
     <row r="2" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.7">
       <c r="A2" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="D2" s="48"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="50" t="s">
-        <v>45</v>
-      </c>
-      <c r="G2" s="51"/>
+        <v>38</v>
+      </c>
+      <c r="D2" s="38"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="40" t="s">
+        <v>39</v>
+      </c>
+      <c r="G2" s="41"/>
     </row>
     <row r="3" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.7">
       <c r="A3" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="B3" s="52" t="s">
-        <v>47</v>
-      </c>
-      <c r="C3" s="53"/>
-      <c r="D3" s="54"/>
+        <v>40</v>
+      </c>
+      <c r="B3" s="42" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="43"/>
+      <c r="D3" s="44"/>
       <c r="F3" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="G3" s="52" t="s">
-        <v>47</v>
-      </c>
-      <c r="H3" s="53"/>
-      <c r="I3" s="54"/>
+        <v>40</v>
+      </c>
+      <c r="G3" s="42" t="s">
+        <v>41</v>
+      </c>
+      <c r="H3" s="43"/>
+      <c r="I3" s="44"/>
     </row>
     <row r="4" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.7">
       <c r="A4" s="19" t="s">
-        <v>60</v>
-      </c>
-      <c r="B4" s="32" t="s">
-        <v>73</v>
-      </c>
-      <c r="C4" s="33"/>
-      <c r="D4" s="34"/>
+        <v>54</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" s="31"/>
+      <c r="D4" s="32"/>
       <c r="F4" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="G4" s="33" t="s">
         <v>68</v>
       </c>
-      <c r="G4" s="35" t="s">
-        <v>74</v>
-      </c>
-      <c r="H4" s="36"/>
-      <c r="I4" s="37"/>
+      <c r="H4" s="34"/>
+      <c r="I4" s="35"/>
     </row>
     <row r="5" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.7">
       <c r="A5" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="B5" s="32" t="s">
-        <v>65</v>
-      </c>
-      <c r="C5" s="33"/>
-      <c r="D5" s="34"/>
+        <v>55</v>
+      </c>
+      <c r="B5" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="C5" s="31"/>
+      <c r="D5" s="32"/>
       <c r="F5" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="G5" s="33" t="s">
         <v>69</v>
       </c>
-      <c r="G5" s="35" t="s">
-        <v>75</v>
-      </c>
-      <c r="H5" s="36"/>
-      <c r="I5" s="37"/>
+      <c r="H5" s="34"/>
+      <c r="I5" s="35"/>
     </row>
     <row r="6" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.7">
       <c r="A6" s="19" t="s">
-        <v>67</v>
-      </c>
-      <c r="B6" s="32" t="s">
-        <v>66</v>
-      </c>
-      <c r="C6" s="33"/>
-      <c r="D6" s="34"/>
+        <v>61</v>
+      </c>
+      <c r="B6" s="30" t="s">
+        <v>60</v>
+      </c>
+      <c r="C6" s="31"/>
+      <c r="D6" s="32"/>
       <c r="F6" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="G6" s="35" t="s">
-        <v>63</v>
-      </c>
-      <c r="H6" s="36"/>
-      <c r="I6" s="37"/>
+        <v>64</v>
+      </c>
+      <c r="G6" s="33" t="s">
+        <v>57</v>
+      </c>
+      <c r="H6" s="34"/>
+      <c r="I6" s="35"/>
     </row>
     <row r="7" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.7">
       <c r="A7" s="19"/>
-      <c r="B7" s="32"/>
-      <c r="C7" s="33"/>
-      <c r="D7" s="34"/>
+      <c r="B7" s="30"/>
+      <c r="C7" s="31"/>
+      <c r="D7" s="32"/>
       <c r="F7" s="19" t="s">
-        <v>71</v>
-      </c>
-      <c r="G7" s="35" t="s">
-        <v>64</v>
-      </c>
-      <c r="H7" s="36"/>
-      <c r="I7" s="37"/>
+        <v>65</v>
+      </c>
+      <c r="G7" s="33" t="s">
+        <v>58</v>
+      </c>
+      <c r="H7" s="34"/>
+      <c r="I7" s="35"/>
     </row>
     <row r="8" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.7">
       <c r="A8" s="19"/>
-      <c r="B8" s="32"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="34"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="31"/>
+      <c r="D8" s="32"/>
       <c r="F8" s="19"/>
-      <c r="G8" s="35"/>
-      <c r="H8" s="36"/>
-      <c r="I8" s="37"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="34"/>
+      <c r="I8" s="35"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.65">
-      <c r="A10" s="38" t="s">
+      <c r="A10" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B10" s="39"/>
-      <c r="C10" s="39"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="40"/>
+      <c r="B10" s="49"/>
+      <c r="C10" s="49"/>
+      <c r="D10" s="49"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="50"/>
       <c r="I10" s="21"/>
       <c r="J10" s="22"/>
       <c r="K10" s="22"/>
@@ -1387,16 +1493,16 @@
       <c r="A12" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="B12" s="41" t="s">
-        <v>51</v>
-      </c>
-      <c r="C12" s="42"/>
-      <c r="D12" s="42"/>
+      <c r="B12" s="51" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" s="52"/>
+      <c r="D12" s="52"/>
       <c r="E12" s="24" t="s">
         <v>11</v>
       </c>
       <c r="F12" s="25" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="I12" s="21"/>
     </row>
@@ -1404,16 +1510,16 @@
       <c r="A13" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="B13" s="41" t="s">
-        <v>48</v>
-      </c>
-      <c r="C13" s="42"/>
-      <c r="D13" s="42"/>
+      <c r="B13" s="51" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" s="52"/>
+      <c r="D13" s="52"/>
       <c r="E13" s="24" t="s">
         <v>3</v>
       </c>
       <c r="F13" s="25" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="I13" s="21"/>
     </row>
@@ -1421,9 +1527,9 @@
       <c r="A14" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="B14" s="43"/>
-      <c r="C14" s="44"/>
-      <c r="D14" s="45"/>
+      <c r="B14" s="45"/>
+      <c r="C14" s="46"/>
+      <c r="D14" s="47"/>
       <c r="E14" s="24" t="s">
         <v>10</v>
       </c>
@@ -1434,81 +1540,81 @@
       <c r="I15" s="21"/>
     </row>
     <row r="16" spans="1:12" ht="25.05" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A16" s="29" t="s">
+      <c r="A16" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="B16" s="30" t="s">
+      <c r="B16" s="54" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="30"/>
-      <c r="D16" s="29" t="s">
+      <c r="C16" s="54"/>
+      <c r="D16" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="E16" s="29" t="s">
+      <c r="E16" s="53" t="s">
         <v>8</v>
       </c>
-      <c r="F16" s="31" t="s">
+      <c r="F16" s="55" t="s">
         <v>9</v>
       </c>
       <c r="I16" s="21"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.65">
-      <c r="A17" s="29"/>
+      <c r="A17" s="53"/>
       <c r="B17" s="27" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C17" s="27" t="s">
-        <v>50</v>
-      </c>
-      <c r="D17" s="29"/>
-      <c r="E17" s="29"/>
-      <c r="F17" s="31"/>
+        <v>44</v>
+      </c>
+      <c r="D17" s="53"/>
+      <c r="E17" s="53"/>
+      <c r="F17" s="55"/>
       <c r="I17" s="21"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A18" s="25" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="B18" s="25" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="C18" s="25">
         <v>-4</v>
       </c>
       <c r="D18" s="25" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="E18" s="25"/>
       <c r="F18" s="25"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A19" s="25" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="B19" s="25" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C19" s="25">
         <v>20</v>
       </c>
       <c r="D19" s="25" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="E19" s="25"/>
       <c r="F19" s="25"/>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A20" s="25" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="B20" s="25" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="C20" s="25">
         <v>-36</v>
       </c>
       <c r="D20" s="25" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="E20" s="25"/>
       <c r="F20" s="25"/>
@@ -1519,16 +1625,16 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A21" s="25" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="B21" s="25" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="C21" s="25">
         <v>30</v>
       </c>
       <c r="D21" s="25" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="E21" s="25"/>
       <c r="F21" s="25"/>
@@ -1539,16 +1645,16 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A22" s="25" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="B22" s="25" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="C22" s="25">
         <v>-1</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="E22" s="25"/>
       <c r="F22" s="25"/>
@@ -1559,16 +1665,16 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A23" s="25" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="B23" s="25" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="C23" s="25">
         <v>13</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="E23" s="25"/>
       <c r="F23" s="25"/>
@@ -1579,7 +1685,7 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A24" s="25" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B24" s="25"/>
       <c r="C24" s="25"/>
@@ -1593,7 +1699,7 @@
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A25" s="25" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B25" s="25"/>
       <c r="C25" s="25"/>
@@ -1607,7 +1713,7 @@
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A26" s="25" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="B26" s="25"/>
       <c r="C26" s="25"/>
@@ -1618,7 +1724,7 @@
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A27" s="25" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B27" s="25"/>
       <c r="C27" s="25"/>
@@ -1632,7 +1738,7 @@
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A28" s="25" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B28" s="25"/>
       <c r="C28" s="25"/>
@@ -1642,7 +1748,7 @@
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A29" s="25" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B29" s="25"/>
       <c r="C29" s="25"/>
@@ -1652,7 +1758,7 @@
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A30" s="25" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B30" s="25"/>
       <c r="C30" s="25"/>
@@ -1705,20 +1811,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="F16:F17"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="G3:I3"/>
     <mergeCell ref="B7:D7"/>
     <mergeCell ref="G7:I7"/>
     <mergeCell ref="B8:D8"/>
@@ -1729,6 +1821,20 @@
     <mergeCell ref="G5:I5"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="G6:I6"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="G3:I3"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="F16:F17"/>
+    <mergeCell ref="A16:A17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1752,134 +1858,134 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="46" t="s">
-        <v>43</v>
-      </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="47"/>
+      <c r="A1" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="37"/>
     </row>
     <row r="2" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.7">
       <c r="A2" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="D2" s="48"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="50" t="s">
-        <v>45</v>
-      </c>
-      <c r="G2" s="51"/>
+        <v>38</v>
+      </c>
+      <c r="D2" s="38"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="40" t="s">
+        <v>39</v>
+      </c>
+      <c r="G2" s="41"/>
     </row>
     <row r="3" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.7">
       <c r="A3" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="B3" s="52" t="s">
-        <v>47</v>
-      </c>
-      <c r="C3" s="53"/>
-      <c r="D3" s="54"/>
+        <v>40</v>
+      </c>
+      <c r="B3" s="42" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="43"/>
+      <c r="D3" s="44"/>
       <c r="F3" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="G3" s="52" t="s">
-        <v>47</v>
-      </c>
-      <c r="H3" s="53"/>
-      <c r="I3" s="54"/>
+        <v>40</v>
+      </c>
+      <c r="G3" s="42" t="s">
+        <v>41</v>
+      </c>
+      <c r="H3" s="43"/>
+      <c r="I3" s="44"/>
     </row>
     <row r="4" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.7">
       <c r="A4" s="19" t="s">
-        <v>60</v>
-      </c>
-      <c r="B4" s="32" t="s">
-        <v>73</v>
-      </c>
-      <c r="C4" s="33"/>
-      <c r="D4" s="34"/>
+        <v>54</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" s="31"/>
+      <c r="D4" s="32"/>
       <c r="F4" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="G4" s="33" t="s">
         <v>68</v>
       </c>
-      <c r="G4" s="35" t="s">
-        <v>74</v>
-      </c>
-      <c r="H4" s="36"/>
-      <c r="I4" s="37"/>
+      <c r="H4" s="34"/>
+      <c r="I4" s="35"/>
     </row>
     <row r="5" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.7">
       <c r="A5" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="B5" s="32" t="s">
-        <v>65</v>
-      </c>
-      <c r="C5" s="33"/>
-      <c r="D5" s="34"/>
+        <v>55</v>
+      </c>
+      <c r="B5" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="C5" s="31"/>
+      <c r="D5" s="32"/>
       <c r="F5" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="G5" s="33" t="s">
         <v>69</v>
       </c>
-      <c r="G5" s="35" t="s">
-        <v>75</v>
-      </c>
-      <c r="H5" s="36"/>
-      <c r="I5" s="37"/>
+      <c r="H5" s="34"/>
+      <c r="I5" s="35"/>
     </row>
     <row r="6" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.7">
       <c r="A6" s="19" t="s">
-        <v>67</v>
-      </c>
-      <c r="B6" s="32" t="s">
-        <v>66</v>
-      </c>
-      <c r="C6" s="33"/>
-      <c r="D6" s="34"/>
+        <v>61</v>
+      </c>
+      <c r="B6" s="30" t="s">
+        <v>60</v>
+      </c>
+      <c r="C6" s="31"/>
+      <c r="D6" s="32"/>
       <c r="F6" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="G6" s="35" t="s">
-        <v>63</v>
-      </c>
-      <c r="H6" s="36"/>
-      <c r="I6" s="37"/>
+        <v>64</v>
+      </c>
+      <c r="G6" s="33" t="s">
+        <v>57</v>
+      </c>
+      <c r="H6" s="34"/>
+      <c r="I6" s="35"/>
     </row>
     <row r="7" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.7">
       <c r="A7" s="19"/>
-      <c r="B7" s="32"/>
-      <c r="C7" s="33"/>
-      <c r="D7" s="34"/>
+      <c r="B7" s="30"/>
+      <c r="C7" s="31"/>
+      <c r="D7" s="32"/>
       <c r="F7" s="19" t="s">
-        <v>71</v>
-      </c>
-      <c r="G7" s="35" t="s">
-        <v>64</v>
-      </c>
-      <c r="H7" s="36"/>
-      <c r="I7" s="37"/>
+        <v>65</v>
+      </c>
+      <c r="G7" s="33" t="s">
+        <v>58</v>
+      </c>
+      <c r="H7" s="34"/>
+      <c r="I7" s="35"/>
     </row>
     <row r="8" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.7">
       <c r="A8" s="19"/>
-      <c r="B8" s="32"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="34"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="31"/>
+      <c r="D8" s="32"/>
       <c r="F8" s="19"/>
-      <c r="G8" s="35"/>
-      <c r="H8" s="36"/>
-      <c r="I8" s="37"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="34"/>
+      <c r="I8" s="35"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.65">
-      <c r="A10" s="38" t="s">
+      <c r="A10" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B10" s="39"/>
-      <c r="C10" s="39"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="40"/>
+      <c r="B10" s="49"/>
+      <c r="C10" s="49"/>
+      <c r="D10" s="49"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="50"/>
       <c r="I10" s="21"/>
       <c r="J10" s="22"/>
       <c r="K10" s="22"/>
@@ -1893,16 +1999,16 @@
       <c r="A12" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="B12" s="41" t="s">
-        <v>52</v>
-      </c>
-      <c r="C12" s="42"/>
-      <c r="D12" s="42"/>
+      <c r="B12" s="51" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" s="52"/>
+      <c r="D12" s="52"/>
       <c r="E12" s="24" t="s">
         <v>11</v>
       </c>
       <c r="F12" s="25" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="I12" s="21"/>
     </row>
@@ -1910,16 +2016,16 @@
       <c r="A13" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="B13" s="41" t="s">
-        <v>48</v>
-      </c>
-      <c r="C13" s="42"/>
-      <c r="D13" s="42"/>
+      <c r="B13" s="51" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" s="52"/>
+      <c r="D13" s="52"/>
       <c r="E13" s="24" t="s">
         <v>3</v>
       </c>
       <c r="F13" s="25" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="I13" s="21"/>
     </row>
@@ -1927,9 +2033,9 @@
       <c r="A14" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="B14" s="43"/>
-      <c r="C14" s="44"/>
-      <c r="D14" s="45"/>
+      <c r="B14" s="45"/>
+      <c r="C14" s="46"/>
+      <c r="D14" s="47"/>
       <c r="E14" s="24" t="s">
         <v>10</v>
       </c>
@@ -1940,81 +2046,81 @@
       <c r="I15" s="21"/>
     </row>
     <row r="16" spans="1:12" ht="25.05" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A16" s="29" t="s">
+      <c r="A16" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="B16" s="30" t="s">
+      <c r="B16" s="54" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="30"/>
-      <c r="D16" s="29" t="s">
+      <c r="C16" s="54"/>
+      <c r="D16" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="E16" s="29" t="s">
+      <c r="E16" s="53" t="s">
         <v>8</v>
       </c>
-      <c r="F16" s="31" t="s">
+      <c r="F16" s="55" t="s">
         <v>9</v>
       </c>
       <c r="I16" s="21"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.65">
-      <c r="A17" s="29"/>
+      <c r="A17" s="53"/>
       <c r="B17" s="27" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="C17" s="27" t="s">
-        <v>50</v>
-      </c>
-      <c r="D17" s="29"/>
-      <c r="E17" s="29"/>
-      <c r="F17" s="31"/>
+        <v>44</v>
+      </c>
+      <c r="D17" s="53"/>
+      <c r="E17" s="53"/>
+      <c r="F17" s="55"/>
       <c r="I17" s="21"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A18" s="25" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="B18" s="25" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="C18" s="25">
         <v>-19</v>
       </c>
       <c r="D18" s="25" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="E18" s="25"/>
       <c r="F18" s="25"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A19" s="25" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B19" s="25" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="C19" s="25">
         <v>20</v>
       </c>
       <c r="D19" s="25" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="E19" s="25"/>
       <c r="F19" s="25"/>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A20" s="25" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="B20" s="25" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="C20" s="25">
         <v>-52</v>
       </c>
       <c r="D20" s="25" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="E20" s="25"/>
       <c r="F20" s="25"/>
@@ -2025,16 +2131,16 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A21" s="25" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="B21" s="25" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="C21" s="25">
         <v>78</v>
       </c>
       <c r="D21" s="25" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="E21" s="25"/>
       <c r="F21" s="25"/>
@@ -2045,16 +2151,16 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A22" s="25" t="s">
-        <v>95</v>
-      </c>
-      <c r="B22" s="55">
+        <v>89</v>
+      </c>
+      <c r="B22" s="29">
         <v>12345</v>
       </c>
       <c r="C22" s="25">
         <v>-1</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="E22" s="25"/>
       <c r="F22" s="25"/>
@@ -2065,16 +2171,16 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A23" s="25" t="s">
+        <v>90</v>
+      </c>
+      <c r="B23" s="25" t="s">
         <v>96</v>
-      </c>
-      <c r="B23" s="25" t="s">
-        <v>102</v>
       </c>
       <c r="C23" s="25">
         <v>3</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="E23" s="25"/>
       <c r="F23" s="25"/>
@@ -2085,7 +2191,7 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A24" s="25" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B24" s="25"/>
       <c r="C24" s="25"/>
@@ -2099,7 +2205,7 @@
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A25" s="25" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B25" s="25"/>
       <c r="C25" s="25"/>
@@ -2113,7 +2219,7 @@
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A26" s="25" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="B26" s="25"/>
       <c r="C26" s="25"/>
@@ -2124,7 +2230,7 @@
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A27" s="25" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B27" s="25"/>
       <c r="C27" s="25"/>
@@ -2138,7 +2244,7 @@
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A28" s="25" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B28" s="25"/>
       <c r="C28" s="25"/>
@@ -2148,7 +2254,7 @@
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A29" s="25" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B29" s="25"/>
       <c r="C29" s="25"/>
@@ -2158,7 +2264,7 @@
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A30" s="25" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B30" s="25"/>
       <c r="C30" s="25"/>
@@ -2211,13 +2317,11 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="G4:I4"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="G3:I3"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="F16:F17"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="G5:I5"/>
@@ -2230,11 +2334,13 @@
     <mergeCell ref="A10:F10"/>
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="B13:D13"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="F16:F17"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="G4:I4"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="G3:I3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2242,16 +2348,18 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0F057A9-52F5-E645-A881-0DE90C7BD7B5}">
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:O37"/>
   <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="24" x14ac:dyDescent="0.65"/>
   <cols>
     <col min="1" max="1" width="17.69921875" style="20" customWidth="1"/>
     <col min="2" max="2" width="41.19921875" style="20" customWidth="1"/>
     <col min="3" max="3" width="26.296875" style="20" customWidth="1"/>
-    <col min="4" max="4" width="23.5" style="20" customWidth="1"/>
-    <col min="5" max="5" width="20.19921875" style="20" customWidth="1"/>
-    <col min="6" max="6" width="25.19921875" style="20" customWidth="1"/>
-    <col min="7" max="9" width="10.796875" style="20"/>
+    <col min="4" max="4" width="27.59765625" style="20" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25" style="20" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.69921875" style="20" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="50.296875" style="20" customWidth="1"/>
+    <col min="8" max="8" width="22.69921875" style="20" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.796875" style="20"/>
     <col min="10" max="10" width="15.296875" style="20" customWidth="1"/>
     <col min="11" max="11" width="10.796875" style="20"/>
     <col min="12" max="12" width="16.5" style="20" customWidth="1"/>
@@ -2259,106 +2367,131 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="46" t="s">
-        <v>43</v>
-      </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="47"/>
+      <c r="A1" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="37"/>
     </row>
     <row r="2" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.7">
       <c r="A2" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="D2" s="48"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="50" t="s">
-        <v>45</v>
-      </c>
-      <c r="G2" s="51"/>
+        <v>38</v>
+      </c>
+      <c r="D2" s="38"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="57" t="s">
+        <v>39</v>
+      </c>
+      <c r="G2" s="57"/>
     </row>
     <row r="3" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.7">
       <c r="A3" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="B3" s="52" t="s">
-        <v>47</v>
-      </c>
-      <c r="C3" s="53"/>
-      <c r="D3" s="54"/>
-      <c r="F3" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="G3" s="52" t="s">
-        <v>47</v>
-      </c>
-      <c r="H3" s="53"/>
-      <c r="I3" s="54"/>
+        <v>40</v>
+      </c>
+      <c r="B3" s="42" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="43"/>
+      <c r="D3" s="44"/>
+      <c r="F3" s="58" t="s">
+        <v>40</v>
+      </c>
+      <c r="G3" s="59" t="s">
+        <v>41</v>
+      </c>
+      <c r="I3" s="21"/>
     </row>
     <row r="4" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.7">
-      <c r="A4" s="19"/>
-      <c r="B4" s="32"/>
-      <c r="C4" s="33"/>
-      <c r="D4" s="34"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="35"/>
-      <c r="H4" s="36"/>
-      <c r="I4" s="37"/>
+      <c r="A4" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="C4" s="31"/>
+      <c r="D4" s="32"/>
+      <c r="F4" s="60" t="s">
+        <v>63</v>
+      </c>
+      <c r="G4" s="61" t="s">
+        <v>100</v>
+      </c>
+      <c r="I4" s="21"/>
     </row>
     <row r="5" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.7">
-      <c r="A5" s="19"/>
-      <c r="B5" s="32"/>
-      <c r="C5" s="33"/>
-      <c r="D5" s="34"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="35"/>
-      <c r="H5" s="36"/>
-      <c r="I5" s="37"/>
+      <c r="A5" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5" s="30" t="s">
+        <v>98</v>
+      </c>
+      <c r="C5" s="31"/>
+      <c r="D5" s="32"/>
+      <c r="F5" s="60" t="s">
+        <v>64</v>
+      </c>
+      <c r="G5" s="61" t="s">
+        <v>101</v>
+      </c>
+      <c r="I5" s="21"/>
     </row>
     <row r="6" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.7">
-      <c r="A6" s="19"/>
-      <c r="B6" s="32"/>
-      <c r="C6" s="33"/>
-      <c r="D6" s="34"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="35"/>
-      <c r="H6" s="36"/>
-      <c r="I6" s="37"/>
+      <c r="A6" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" s="30" t="s">
+        <v>99</v>
+      </c>
+      <c r="C6" s="31"/>
+      <c r="D6" s="32"/>
+      <c r="F6" s="60" t="s">
+        <v>65</v>
+      </c>
+      <c r="G6" s="61" t="s">
+        <v>104</v>
+      </c>
+      <c r="I6" s="21"/>
     </row>
     <row r="7" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.7">
-      <c r="A7" s="19"/>
-      <c r="B7" s="32"/>
-      <c r="C7" s="33"/>
-      <c r="D7" s="34"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="35"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="37"/>
+      <c r="A7" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="B7" s="30" t="s">
+        <v>102</v>
+      </c>
+      <c r="C7" s="31"/>
+      <c r="D7" s="32"/>
+      <c r="F7" s="60"/>
+      <c r="G7" s="61"/>
+      <c r="I7" s="21"/>
     </row>
     <row r="8" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.7">
       <c r="A8" s="19"/>
-      <c r="B8" s="32"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="34"/>
-      <c r="F8" s="19"/>
-      <c r="G8" s="35"/>
-      <c r="H8" s="36"/>
-      <c r="I8" s="37"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="31"/>
+      <c r="D8" s="32"/>
+      <c r="F8" s="60"/>
+      <c r="G8" s="61"/>
+      <c r="I8" s="21"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.65">
+      <c r="I9" s="21"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.65">
-      <c r="A10" s="38" t="s">
+      <c r="A10" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B10" s="39"/>
-      <c r="C10" s="39"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="40"/>
+      <c r="B10" s="49"/>
+      <c r="C10" s="49"/>
+      <c r="D10" s="49"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="50"/>
       <c r="I10" s="21"/>
       <c r="J10" s="22"/>
       <c r="K10" s="22"/>
@@ -2366,39 +2499,37 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.65">
       <c r="F11" s="23"/>
-      <c r="I11" s="21"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A12" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="B12" s="41" t="s">
-        <v>54</v>
-      </c>
-      <c r="C12" s="42"/>
-      <c r="D12" s="42"/>
+      <c r="B12" s="51" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" s="52"/>
+      <c r="D12" s="52"/>
       <c r="E12" s="24" t="s">
         <v>11</v>
       </c>
       <c r="F12" s="25" t="s">
-        <v>58</v>
-      </c>
-      <c r="I12" s="21"/>
+        <v>52</v>
+      </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.65">
       <c r="A13" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="B13" s="41" t="s">
-        <v>56</v>
-      </c>
-      <c r="C13" s="42"/>
-      <c r="D13" s="42"/>
+      <c r="B13" s="51" t="s">
+        <v>50</v>
+      </c>
+      <c r="C13" s="52"/>
+      <c r="D13" s="52"/>
       <c r="E13" s="24" t="s">
         <v>3</v>
       </c>
       <c r="F13" s="25" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="I13" s="21"/>
     </row>
@@ -2406,9 +2537,9 @@
       <c r="A14" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="B14" s="43"/>
-      <c r="C14" s="44"/>
-      <c r="D14" s="45"/>
+      <c r="B14" s="45"/>
+      <c r="C14" s="46"/>
+      <c r="D14" s="47"/>
       <c r="E14" s="24" t="s">
         <v>10</v>
       </c>
@@ -2419,264 +2550,362 @@
       <c r="I15" s="21"/>
     </row>
     <row r="16" spans="1:12" ht="25.05" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A16" s="29" t="s">
+      <c r="A16" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="B16" s="30" t="s">
+      <c r="B16" s="54" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="30"/>
-      <c r="D16" s="29" t="s">
-        <v>7</v>
-      </c>
-      <c r="E16" s="29" t="s">
-        <v>8</v>
-      </c>
-      <c r="F16" s="31" t="s">
+      <c r="C16" s="54"/>
+      <c r="D16" s="53" t="s">
+        <v>111</v>
+      </c>
+      <c r="E16" s="53" t="s">
+        <v>112</v>
+      </c>
+      <c r="F16" s="55" t="s">
         <v>9</v>
       </c>
-      <c r="I16" s="21"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.65">
-      <c r="A17" s="29"/>
+      <c r="G16" s="53" t="s">
+        <v>113</v>
+      </c>
+      <c r="H16" s="53" t="s">
+        <v>114</v>
+      </c>
+      <c r="I16" s="55" t="s">
+        <v>9</v>
+      </c>
+      <c r="L16" s="21"/>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.65">
+      <c r="A17" s="53"/>
       <c r="B17" s="27" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C17" s="27" t="s">
-        <v>57</v>
-      </c>
-      <c r="D17" s="29"/>
-      <c r="E17" s="29"/>
-      <c r="F17" s="31"/>
-      <c r="I17" s="21"/>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.65">
+        <v>51</v>
+      </c>
+      <c r="D17" s="53"/>
+      <c r="E17" s="53"/>
+      <c r="F17" s="55"/>
+      <c r="G17" s="53"/>
+      <c r="H17" s="53"/>
+      <c r="I17" s="55"/>
+      <c r="L17" s="21"/>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.65">
       <c r="A18" s="25" t="s">
-        <v>30</v>
-      </c>
-      <c r="B18" s="25"/>
-      <c r="C18" s="25"/>
-      <c r="D18" s="25"/>
+        <v>103</v>
+      </c>
+      <c r="B18" s="25" t="s">
+        <v>118</v>
+      </c>
+      <c r="C18" s="25" t="s">
+        <v>119</v>
+      </c>
+      <c r="D18" s="25">
+        <v>250</v>
+      </c>
       <c r="E18" s="25"/>
       <c r="F18" s="25"/>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.65">
+      <c r="G18" s="25">
+        <v>250</v>
+      </c>
+      <c r="H18" s="25"/>
+      <c r="I18" s="25"/>
+      <c r="L18" s="21"/>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.65">
       <c r="A19" s="25" t="s">
-        <v>31</v>
-      </c>
-      <c r="B19" s="25"/>
-      <c r="C19" s="25"/>
+        <v>105</v>
+      </c>
+      <c r="B19" s="62" t="s">
+        <v>121</v>
+      </c>
+      <c r="C19" s="25" t="s">
+        <v>122</v>
+      </c>
+      <c r="D19" s="25">
+        <v>300</v>
+      </c>
       <c r="E19" s="25"/>
       <c r="F19" s="25"/>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.65">
+      <c r="G19" s="25">
+        <v>300</v>
+      </c>
+      <c r="H19" s="25"/>
+      <c r="I19" s="25"/>
+      <c r="L19" s="21"/>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.65">
       <c r="A20" s="25" t="s">
-        <v>32</v>
-      </c>
-      <c r="B20" s="25"/>
-      <c r="C20" s="25"/>
-      <c r="D20" s="25"/>
+        <v>106</v>
+      </c>
+      <c r="B20" s="62" t="s">
+        <v>123</v>
+      </c>
+      <c r="C20" s="25" t="s">
+        <v>124</v>
+      </c>
+      <c r="D20" s="25">
+        <v>500</v>
+      </c>
       <c r="E20" s="25"/>
       <c r="F20" s="25"/>
-      <c r="I20" s="21"/>
-      <c r="J20" s="21"/>
-      <c r="K20" s="21"/>
+      <c r="G20" s="25">
+        <v>500</v>
+      </c>
+      <c r="H20" s="25"/>
+      <c r="I20" s="25"/>
       <c r="L20" s="21"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.65">
+      <c r="M20" s="21"/>
+      <c r="N20" s="21"/>
+      <c r="O20" s="21"/>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.65">
       <c r="A21" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="B21" s="25"/>
-      <c r="C21" s="25"/>
-      <c r="D21" s="25"/>
+        <v>107</v>
+      </c>
+      <c r="B21" s="62" t="s">
+        <v>127</v>
+      </c>
+      <c r="C21" s="25" t="s">
+        <v>128</v>
+      </c>
+      <c r="D21" s="25">
+        <v>200</v>
+      </c>
       <c r="E21" s="25"/>
       <c r="F21" s="25"/>
-      <c r="I21" s="21"/>
-      <c r="J21" s="21"/>
-      <c r="K21" s="21"/>
-      <c r="L21" s="21"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.65">
+      <c r="G21" s="25">
+        <v>200</v>
+      </c>
+      <c r="H21" s="25"/>
+      <c r="I21" s="25"/>
+      <c r="M21" s="21"/>
+      <c r="N21" s="21"/>
+      <c r="O21" s="21"/>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.65">
       <c r="A22" s="25" t="s">
-        <v>34</v>
-      </c>
-      <c r="B22" s="25"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="25"/>
+        <v>108</v>
+      </c>
+      <c r="B22" s="25" t="s">
+        <v>120</v>
+      </c>
+      <c r="C22" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="D22" s="25" t="s">
+        <v>115</v>
+      </c>
       <c r="E22" s="25"/>
       <c r="F22" s="25"/>
-      <c r="I22" s="21"/>
-      <c r="J22" s="21"/>
-      <c r="K22" s="21"/>
-      <c r="L22" s="21"/>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.65">
+      <c r="G22" s="25" t="s">
+        <v>115</v>
+      </c>
+      <c r="H22" s="25"/>
+      <c r="I22" s="25"/>
+      <c r="M22" s="21"/>
+      <c r="N22" s="21"/>
+      <c r="O22" s="21"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.65">
       <c r="A23" s="25" t="s">
-        <v>35</v>
-      </c>
-      <c r="B23" s="25"/>
-      <c r="C23" s="25"/>
-      <c r="D23" s="25"/>
+        <v>109</v>
+      </c>
+      <c r="B23" s="25" t="s">
+        <v>126</v>
+      </c>
+      <c r="C23" s="25" t="s">
+        <v>130</v>
+      </c>
+      <c r="D23" s="25" t="s">
+        <v>116</v>
+      </c>
       <c r="E23" s="25"/>
       <c r="F23" s="25"/>
-      <c r="I23" s="21"/>
-      <c r="J23" s="21"/>
-      <c r="K23" s="21"/>
+      <c r="G23" s="25" t="s">
+        <v>116</v>
+      </c>
+      <c r="H23" s="25"/>
+      <c r="I23" s="25"/>
       <c r="L23" s="21"/>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.65">
+      <c r="M23" s="21"/>
+      <c r="N23" s="21"/>
+      <c r="O23" s="21"/>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.65">
       <c r="A24" s="25" t="s">
-        <v>36</v>
-      </c>
-      <c r="B24" s="25"/>
-      <c r="C24" s="25"/>
-      <c r="D24" s="25"/>
+        <v>110</v>
+      </c>
+      <c r="B24" s="25" t="s">
+        <v>125</v>
+      </c>
+      <c r="C24" s="25" t="s">
+        <v>131</v>
+      </c>
+      <c r="D24" s="25" t="s">
+        <v>117</v>
+      </c>
       <c r="E24" s="25"/>
       <c r="F24" s="25"/>
-      <c r="I24" s="21"/>
-      <c r="J24" s="21"/>
-      <c r="K24" s="21"/>
+      <c r="G24" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="H24" s="25"/>
+      <c r="I24" s="25"/>
       <c r="L24" s="21"/>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.65">
+      <c r="M24" s="21"/>
+      <c r="N24" s="21"/>
+      <c r="O24" s="21"/>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.65">
       <c r="A25" s="25" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B25" s="25"/>
       <c r="C25" s="25"/>
       <c r="D25" s="25"/>
       <c r="E25" s="25"/>
       <c r="F25" s="25"/>
-      <c r="I25" s="21"/>
-      <c r="J25" s="21"/>
-      <c r="K25" s="21"/>
+      <c r="G25" s="25"/>
+      <c r="H25" s="25"/>
+      <c r="I25" s="25"/>
       <c r="L25" s="21"/>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.65">
+      <c r="M25" s="21"/>
+      <c r="N25" s="21"/>
+      <c r="O25" s="21"/>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.65">
       <c r="A26" s="25" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="B26" s="25"/>
       <c r="C26" s="25"/>
       <c r="D26" s="25"/>
       <c r="E26" s="25"/>
       <c r="F26" s="25"/>
-      <c r="I26" s="21"/>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.65">
+      <c r="G26" s="25"/>
+      <c r="H26" s="25"/>
+      <c r="I26" s="25"/>
+      <c r="L26" s="21"/>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.65">
       <c r="A27" s="25" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B27" s="25"/>
       <c r="C27" s="25"/>
       <c r="D27" s="25"/>
       <c r="E27" s="25"/>
       <c r="F27" s="25"/>
-      <c r="I27" s="21"/>
-      <c r="J27" s="21"/>
-      <c r="K27" s="21"/>
+      <c r="G27" s="25"/>
+      <c r="H27" s="25"/>
+      <c r="I27" s="25"/>
       <c r="L27" s="21"/>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.65">
+      <c r="M27" s="21"/>
+      <c r="N27" s="21"/>
+      <c r="O27" s="21"/>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.65">
       <c r="A28" s="25" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B28" s="25"/>
       <c r="C28" s="25"/>
       <c r="D28" s="25"/>
       <c r="E28" s="25"/>
       <c r="F28" s="25"/>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.65">
+      <c r="G28" s="25"/>
+      <c r="H28" s="25"/>
+      <c r="I28" s="25"/>
+      <c r="L28" s="21"/>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.65">
       <c r="A29" s="25" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B29" s="25"/>
       <c r="C29" s="25"/>
       <c r="D29" s="25"/>
       <c r="E29" s="25"/>
       <c r="F29" s="25"/>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.65">
+      <c r="G29" s="25"/>
+      <c r="H29" s="25"/>
+      <c r="I29" s="25"/>
+      <c r="L29" s="21"/>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.65">
       <c r="A30" s="25" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B30" s="25"/>
       <c r="C30" s="25"/>
       <c r="D30" s="25"/>
       <c r="E30" s="25"/>
       <c r="F30" s="25"/>
-      <c r="I30" s="21"/>
-      <c r="J30" s="21"/>
-      <c r="K30" s="21"/>
+      <c r="G30" s="25"/>
+      <c r="H30" s="25"/>
+      <c r="I30" s="25"/>
       <c r="L30" s="21"/>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.65">
-      <c r="I31" s="21"/>
+      <c r="M30" s="21"/>
+      <c r="N30" s="21"/>
+      <c r="O30" s="21"/>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.65">
       <c r="J31" s="21"/>
       <c r="K31" s="21"/>
       <c r="L31" s="21"/>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.65">
-      <c r="I32" s="21"/>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.65">
       <c r="J32" s="21"/>
       <c r="K32" s="21"/>
       <c r="L32" s="21"/>
     </row>
-    <row r="33" spans="9:12" x14ac:dyDescent="0.65">
-      <c r="I33" s="21"/>
+    <row r="33" spans="10:12" x14ac:dyDescent="0.65">
       <c r="J33" s="21"/>
       <c r="K33" s="21"/>
       <c r="L33" s="21"/>
     </row>
-    <row r="34" spans="9:12" x14ac:dyDescent="0.65">
-      <c r="I34" s="21"/>
+    <row r="34" spans="10:12" x14ac:dyDescent="0.65">
       <c r="J34" s="21"/>
       <c r="K34" s="21"/>
       <c r="L34" s="21"/>
     </row>
-    <row r="35" spans="9:12" x14ac:dyDescent="0.65">
-      <c r="I35" s="21"/>
+    <row r="35" spans="10:12" x14ac:dyDescent="0.65">
       <c r="J35" s="21"/>
       <c r="K35" s="21"/>
       <c r="L35" s="21"/>
     </row>
-    <row r="36" spans="9:12" x14ac:dyDescent="0.65">
-      <c r="I36" s="21"/>
-    </row>
-    <row r="37" spans="9:12" x14ac:dyDescent="0.65">
-      <c r="I37" s="21"/>
+    <row r="37" spans="10:12" x14ac:dyDescent="0.65">
       <c r="J37" s="21"/>
       <c r="K37" s="21"/>
       <c r="L37" s="21"/>
     </row>
   </sheetData>
-  <mergeCells count="24">
+  <mergeCells count="21">
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="G16:G17"/>
+    <mergeCell ref="H16:H17"/>
+    <mergeCell ref="I16:I17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="F16:F17"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B13:D13"/>
     <mergeCell ref="B4:D4"/>
-    <mergeCell ref="G4:I4"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="B3:D3"/>
-    <mergeCell ref="G3:I3"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="G5:I5"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="G7:I7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="G8:I8"/>
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="F16:F17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>